<commit_message>
[STYLE] Changed visual search task instructions
</commit_message>
<xml_diff>
--- a/src/instructions/visual_search_task_instructions.xlsx
+++ b/src/instructions/visual_search_task_instructions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\siburmuin\src\begiBrainDemo\instructions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{D13A18B9-AA93-4F1A-9A32-E9C469A51924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91BB155-28F0-4F57-956A-F668786CD1D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>title</t>
   </si>
@@ -119,7 +119,10 @@
     <t>VISUAL SEARCH TEST</t>
   </si>
   <si>
-    <t>Observa las distintas imágenes que aparecerán a continuación.</t>
+    <t>Observa los discos y mantén la mirada en el que tenga una orientación distinta.</t>
+  </si>
+  <si>
+    <t>Pulsa la barra espaciadora para empezar la prueba.</t>
   </si>
 </sst>
 </file>
@@ -546,6 +549,9 @@
       <c r="B2" t="s">
         <v>7</v>
       </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>